<commit_message>
Update mummichog results (sex-adjusted, top 10%), README sections on pathways and validated ROC
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDn5T1yz4TRFaKpaKqad5Y
</commit_message>
<xml_diff>
--- a/results/mummichog/BC_vs_Control/tables/mcg_modularanalysis_BC_vs_Control.xlsx
+++ b/results/mummichog/BC_vs_Control/tables/mcg_modularanalysis_BC_vs_Control.xlsx
@@ -37,25 +37,25 @@
     <t>module_1</t>
   </si>
   <si>
-    <t>Didemethylcitalopram$Demethylcitalopram$3-Methoxytyramine$3-Methoxy-4-hydroxyphenylacetaldehyde$$L-Metanephrine$Norepinephrine$5-Hydroxykynurenamine$L-Adrenaline; (R)-(-)-Adrenaline; (R)-(-)-Epinephrine; (R)-(-)-Epirenamine; (R)-(-)-Adnephrine; 4-[(1R)-1-Hydroxy-2-(methylamino)ethyl]-1,2-benzenediol$3-Methoxy-4-hydroxyphenylglycolaldehyde$$N-Methylphenylethanolamine$noradrenochrome$4,6-Dihydroxyquinoline; Quinoline-4,6-diol$L-Normetanephrine$Citalopram</t>
-  </si>
-  <si>
-    <t>C16609,C16608,C05587,C05581,CE2174,C05588,C00547,C05638,C00788,C05583,CE2173,C03711,CE5538,C05639,C05589,C07572</t>
-  </si>
-  <si>
-    <t>(10, 'Tyrosine metabolism');(3, 'Urea cycle/amino group metabolism');(3, 'Drug metabolism - cytochrome P450')</t>
+    <t>3,4-Dihydroxyphenylacetaldehyde; Protocatechuatealdehyde$L-Normetanephrine$L-Metanephrine$Didemethylcitalopram$Demethylcitalopram$$3-Methoxy-4-hydroxyphenylglycolaldehyde$5-Hydroxykynurenamine$3-Methoxy-4-hydroxyphenylacetaldehyde$3-Methoxytyramine</t>
+  </si>
+  <si>
+    <t>C04043,C05589,C05588,C16609,C16608,C06350,C05583,C05638,C05581,C05587</t>
+  </si>
+  <si>
+    <t>(7, 'Tyrosine metabolism');(2, 'Drug metabolism - cytochrome P450');(1, 'Tryptophan metabolism')</t>
   </si>
   <si>
     <t>module_2</t>
   </si>
   <si>
-    <t>6,7-Dihydrobiopterin$Demethylcitalopram$2-Phenyl-1,3-propanediol monocarbamate$$L-Metanephrine$3-Methoxy-4-hydroxyphenylglycolaldehyde$Dopamine$3-Methoxy-4-hydroxymandelate; Vanillylmandelic acid$Indolepyruvate; Indolepyruvic acid; (Indol-3-yl)pyruvate; Indole-3-pyruvate; 3-(Indol-3-yl)pyruvate$O2'-4a-cyclic-tetrahydrobiopterin$2-Hydroxy-3-(4-hydroxyphenyl)propenoate; 4-Hydroxy-enol-phenylpyruvate$3,4-Dihydroxymandelaldehyde$Didemethylcitalopram$$L-Phenylalanine$3-Methoxytyramine$3-Carbamoyl-2-phenylpropionaldehyde$Phenylpyruvate$5-Hydroxykynurenamine$3-Carbamoyl-2-phenylpropionic acid$Dopaquinone$(-)-Salsolinol; 6,7-Isoquinolinediol, 1,2,3,4-tetrahydro-1-methyl-, (S)-; Salsolinol$Homogentisate$L-Tyrosine$noradrenochrome$4-Hydroxy-5-phenyltetrahydro-1,3-oxazin-2-one$3-O-methyldopa$3-Methoxy-4-hydroxyphenylacetaldehyde$Epinine; Deoxyepinephrine$$Norepinephrine$adrenochrome$3,4-Dihydroxy-L-phenylalanine$3-(4-Hydroxyphenyl)pyruvate$1,2-dehydrosalsolinol$salsolinol 1-carboxylate$Dihydropteridine; 6,7-Dihydropteridine$Homovanillate; Homovanillic acid$salsoline-1-carboxylate$3,4-Dihydroxyphenylacetate; 3,4-Dihydroxyphenylacetic acid; 3,4-Dihydroxyphenyl acetate; 3,4-Dihydroxyphenyl acetic acid; Homoprotocatechuate$adrenochrome o-semiquinone$Dopamine 3-O-sulfate$L-Adrenaline; (R)-(-)-Adrenaline; (R)-(-)-Epinephrine; (R)-(-)-Epirenamine; (R)-(-)-Adnephrine; 4-[(1R)-1-Hydroxy-2-(methylamino)ethyl]-1,2-benzenediol$N-Methylphenylethanolamine$$2-Carboxy-2,3-dihydro-5,6-dihydroxyindole; Leucodopachrome$quinonoid dihydrobiopterin$3,4-Dihydroxymandelate$4,6-Dihydroxyquinoline; Quinoline-4,6-diol$L-Normetanephrine$Citalopram$enol-Phenylpyruvate</t>
-  </si>
-  <si>
-    <t>C00268,C16608,C16586,CE2174,C05588,C05583,C03758,C05584,C00331,CE5236,C05350,C05577,C16609,C06350,C00079,C05587,C16587,C00166,C05638,C16591,C00822,C09642,C00544,C00082,CE5538,C16595,CE2176,C05581,C07453,CE2172,C00547,CE5536,C00355,C01179,CE5629,CE5626,C05649,C05582,CE5627,C01161,CE5541,C13690,C00788,C03711,CE2173,C05604,CE2705,C05580,C05639,C05589,C07572,C02763</t>
-  </si>
-  <si>
-    <t>(38, 'Tyrosine metabolism');(7, 'Drug metabolism - cytochrome P450');(5, 'Biopterin metabolism')</t>
+    <t>L-Normetanephrine$$3,4-Dihydroxymandelaldehyde$N-Methylphenylethanolamine$3,4-Dihydroxyphenylacetate; 3,4-Dihydroxyphenylacetic acid; 3,4-Dihydroxyphenyl acetate; 3,4-Dihydroxyphenyl acetic acid; Homoprotocatechuate$L-Adrenaline; (R)-(-)-Adrenaline; (R)-(-)-Epinephrine; (R)-(-)-Epirenamine; (R)-(-)-Adnephrine; 4-[(1R)-1-Hydroxy-2-(methylamino)ethyl]-1,2-benzenediol$5-Hydroxykynurenamine$3,4-Dihydroxyphenylethyleneglycol$$3,4-Dihydroxyphenylacetaldehyde; Protocatechuatealdehyde$3-Carbamoyl-2-phenylpropionic acid$Norepinephrine$3-Carbamoyl-2-phenylpropionaldehyde$Demethylcitalopram$3-Methoxy-4-hydroxyphenylglycolaldehyde$2-Phenyl-1,3-propanediol monocarbamate$$adrenochrome$3,4-Dihydroxymandelate$3-Methoxy-4-hydroxyphenylethyleneglycol$Homovanillate; Homovanillic acid$3-Methoxy-4-hydroxymandelate; Vanillylmandelic acid$noradrenochrome$3-Methoxytyramine$adrenochrome o-semiquinone$Didemethylcitalopram$L-Metanephrine$4-Hydroxy-5-phenyltetrahydro-1,3-oxazin-2-one$3-Methoxy-4-hydroxyphenylacetaldehyde</t>
+  </si>
+  <si>
+    <t>C05589,C06350,C05577,C03711,C01161,C00788,C05638,C05576,CE2173,C04043,C16591,C00547,C16587,C16608,C05583,C16586,CE2174,CE5536,C05580,C05594,C05582,C05584,CE5538,C05587,CE5541,C16609,C05588,C16595,C05581</t>
+  </si>
+  <si>
+    <t>(21, 'Tyrosine metabolism');(6, 'Drug metabolism - cytochrome P450');(3, 'Urea cycle/amino group metabolism')</t>
   </si>
 </sst>
 </file>
@@ -415,10 +415,10 @@
         <v>6</v>
       </c>
       <c r="B2">
-        <v>0.01518987341772152</v>
+        <v>0.02186528497409326</v>
       </c>
       <c r="C2">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -435,10 +435,10 @@
         <v>10</v>
       </c>
       <c r="B3">
-        <v>0.01924050632911392</v>
+        <v>0.03077720207253886</v>
       </c>
       <c r="C3">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s">
         <v>11</v>

</xml_diff>